<commit_message>
Record initial feature smoke tests
</commit_message>
<xml_diff>
--- a/docs/qa/bellforge-feature-tracker.xlsx
+++ b/docs/qa/bellforge-feature-tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R152788aec37e48e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Stories" sheetId="2" r:id="Rae0bc0d71b374784"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Runs" sheetId="3" r:id="R6e48894760ac470d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defects" sheetId="4" r:id="R7f79362e43c74135"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="5" r:id="R3b3176eab6eb45a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rde54910d3a1f4e51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Stories" sheetId="2" r:id="Re1002ef8d6f34d04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Runs" sheetId="3" r:id="R620b7ece0c594eaf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defects" sheetId="4" r:id="R22c105b773cd4e5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="5" r:id="Re8e4d6e118b847d7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -559,7 +559,7 @@
       </x:c>
       <x:c r="B6" s="4" t="n">
         <x:f>COUNTIF('Feature Stories'!H2:H83,"Not Tested")</x:f>
-        <x:v>82</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="C6" s="1"/>
       <x:c r="D6" s="1"/>
@@ -820,8 +820,8 @@
       <x:c r="J2" s="4" t="str">
         <x:v>P3</x:v>
       </x:c>
-      <x:c r="K2" s="1" t="str"/>
-      <x:c r="L2" s="25" t="str"/>
+      <x:c r="K2" s="1"/>
+      <x:c r="L2" s="25"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="26" t="str">
@@ -854,8 +854,8 @@
       <x:c r="J3" s="4" t="str">
         <x:v>P3</x:v>
       </x:c>
-      <x:c r="K3" s="1" t="str"/>
-      <x:c r="L3" s="25" t="str"/>
+      <x:c r="K3" s="1"/>
+      <x:c r="L3" s="25"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="26" t="str">
@@ -880,16 +880,18 @@
         <x:v>Inventoried</x:v>
       </x:c>
       <x:c r="H4" s="4" t="str">
-        <x:v>Not Tested</x:v>
+        <x:v>Tested</x:v>
       </x:c>
       <x:c r="I4" s="4" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="J4" s="4" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="K4" s="1" t="str"/>
-      <x:c r="L4" s="25" t="str"/>
+      <x:c r="K4" s="1"/>
+      <x:c r="L4" s="25" t="str">
+        <x:v>Smoke tested in browser on localhost:4173 with no console errors.</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="26" t="str">
@@ -914,16 +916,18 @@
         <x:v>Inventoried</x:v>
       </x:c>
       <x:c r="H5" s="4" t="str">
-        <x:v>Not Tested</x:v>
+        <x:v>Tested</x:v>
       </x:c>
       <x:c r="I5" s="4" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="J5" s="4" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="K5" s="1" t="str"/>
-      <x:c r="L5" s="25" t="str"/>
+      <x:c r="K5" s="1"/>
+      <x:c r="L5" s="25" t="str">
+        <x:v>Smoke tested in browser on localhost:4173 with no console errors.</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="26" t="str">
@@ -956,8 +960,8 @@
       <x:c r="J6" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K6" s="1" t="str"/>
-      <x:c r="L6" s="25" t="str"/>
+      <x:c r="K6" s="1"/>
+      <x:c r="L6" s="25"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="26" t="str">
@@ -990,8 +994,8 @@
       <x:c r="J7" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K7" s="1" t="str"/>
-      <x:c r="L7" s="25" t="str"/>
+      <x:c r="K7" s="1"/>
+      <x:c r="L7" s="25"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="26" t="str">
@@ -1024,8 +1028,8 @@
       <x:c r="J8" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K8" s="1" t="str"/>
-      <x:c r="L8" s="25" t="str"/>
+      <x:c r="K8" s="1"/>
+      <x:c r="L8" s="25"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="26" t="str">
@@ -1058,8 +1062,8 @@
       <x:c r="J9" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K9" s="1" t="str"/>
-      <x:c r="L9" s="25" t="str"/>
+      <x:c r="K9" s="1"/>
+      <x:c r="L9" s="25"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="26" t="str">
@@ -1092,8 +1096,8 @@
       <x:c r="J10" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K10" s="1" t="str"/>
-      <x:c r="L10" s="25" t="str"/>
+      <x:c r="K10" s="1"/>
+      <x:c r="L10" s="25"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="26" t="str">
@@ -1126,8 +1130,8 @@
       <x:c r="J11" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K11" s="1" t="str"/>
-      <x:c r="L11" s="25" t="str"/>
+      <x:c r="K11" s="1"/>
+      <x:c r="L11" s="25"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="26" t="str">
@@ -1160,8 +1164,8 @@
       <x:c r="J12" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K12" s="1" t="str"/>
-      <x:c r="L12" s="25" t="str"/>
+      <x:c r="K12" s="1"/>
+      <x:c r="L12" s="25"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="26" t="str">
@@ -1194,8 +1198,8 @@
       <x:c r="J13" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K13" s="1" t="str"/>
-      <x:c r="L13" s="25" t="str"/>
+      <x:c r="K13" s="1"/>
+      <x:c r="L13" s="25"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="26" t="str">
@@ -1228,8 +1232,8 @@
       <x:c r="J14" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K14" s="1" t="str"/>
-      <x:c r="L14" s="25" t="str"/>
+      <x:c r="K14" s="1"/>
+      <x:c r="L14" s="25"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="26" t="str">
@@ -1262,8 +1266,8 @@
       <x:c r="J15" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K15" s="1" t="str"/>
-      <x:c r="L15" s="25" t="str"/>
+      <x:c r="K15" s="1"/>
+      <x:c r="L15" s="25"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="26" t="str">
@@ -1296,8 +1300,8 @@
       <x:c r="J16" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K16" s="1" t="str"/>
-      <x:c r="L16" s="25" t="str"/>
+      <x:c r="K16" s="1"/>
+      <x:c r="L16" s="25"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="26" t="str">
@@ -1330,8 +1334,8 @@
       <x:c r="J17" s="4" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="K17" s="1" t="str"/>
-      <x:c r="L17" s="25" t="str"/>
+      <x:c r="K17" s="1"/>
+      <x:c r="L17" s="25"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="26" t="str">
@@ -1364,8 +1368,8 @@
       <x:c r="J18" s="4" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="K18" s="1" t="str"/>
-      <x:c r="L18" s="25" t="str"/>
+      <x:c r="K18" s="1"/>
+      <x:c r="L18" s="25"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="26" t="str">
@@ -1398,8 +1402,8 @@
       <x:c r="J19" s="4" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="K19" s="1" t="str"/>
-      <x:c r="L19" s="25" t="str"/>
+      <x:c r="K19" s="1"/>
+      <x:c r="L19" s="25"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="26" t="str">
@@ -1432,8 +1436,8 @@
       <x:c r="J20" s="4" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="K20" s="1" t="str"/>
-      <x:c r="L20" s="25" t="str"/>
+      <x:c r="K20" s="1"/>
+      <x:c r="L20" s="25"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="26" t="str">
@@ -1458,16 +1462,18 @@
         <x:v>Inventoried</x:v>
       </x:c>
       <x:c r="H21" s="4" t="str">
-        <x:v>Not Tested</x:v>
+        <x:v>Tested</x:v>
       </x:c>
       <x:c r="I21" s="4" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="J21" s="4" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K21" s="1" t="str"/>
-      <x:c r="L21" s="25" t="str"/>
+      <x:c r="K21" s="1"/>
+      <x:c r="L21" s="25" t="str">
+        <x:v>Smoke tested in browser on localhost:4173 with no console errors.</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="26" t="str">
@@ -1500,8 +1506,8 @@
       <x:c r="J22" s="4" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K22" s="1" t="str"/>
-      <x:c r="L22" s="25" t="str"/>
+      <x:c r="K22" s="1"/>
+      <x:c r="L22" s="25"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="26" t="str">
@@ -1526,16 +1532,18 @@
         <x:v>Inventoried</x:v>
       </x:c>
       <x:c r="H23" s="4" t="str">
-        <x:v>Not Tested</x:v>
+        <x:v>Tested</x:v>
       </x:c>
       <x:c r="I23" s="4" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="J23" s="4" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K23" s="1" t="str"/>
-      <x:c r="L23" s="25" t="str"/>
+      <x:c r="K23" s="1"/>
+      <x:c r="L23" s="25" t="str">
+        <x:v>Smoke tested in browser on localhost:4173 with no console errors.</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="26" t="str">
@@ -1568,8 +1576,8 @@
       <x:c r="J24" s="4" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K24" s="1" t="str"/>
-      <x:c r="L24" s="25" t="str"/>
+      <x:c r="K24" s="1"/>
+      <x:c r="L24" s="25"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="26" t="str">
@@ -1602,8 +1610,8 @@
       <x:c r="J25" s="4" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K25" s="1" t="str"/>
-      <x:c r="L25" s="25" t="str"/>
+      <x:c r="K25" s="1"/>
+      <x:c r="L25" s="25"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="26" t="str">
@@ -1636,8 +1644,8 @@
       <x:c r="J26" s="4" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K26" s="1" t="str"/>
-      <x:c r="L26" s="25" t="str"/>
+      <x:c r="K26" s="1"/>
+      <x:c r="L26" s="25"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="26" t="str">
@@ -1670,8 +1678,8 @@
       <x:c r="J27" s="4" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K27" s="1" t="str"/>
-      <x:c r="L27" s="25" t="str"/>
+      <x:c r="K27" s="1"/>
+      <x:c r="L27" s="25"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="26" t="str">
@@ -1704,8 +1712,8 @@
       <x:c r="J28" s="4" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K28" s="1" t="str"/>
-      <x:c r="L28" s="25" t="str"/>
+      <x:c r="K28" s="1"/>
+      <x:c r="L28" s="25"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="26" t="str">
@@ -1738,8 +1746,8 @@
       <x:c r="J29" s="4" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K29" s="1" t="str"/>
-      <x:c r="L29" s="25" t="str"/>
+      <x:c r="K29" s="1"/>
+      <x:c r="L29" s="25"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="26" t="str">
@@ -1772,8 +1780,8 @@
       <x:c r="J30" s="4" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K30" s="1" t="str"/>
-      <x:c r="L30" s="25" t="str"/>
+      <x:c r="K30" s="1"/>
+      <x:c r="L30" s="25"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="26" t="str">
@@ -1798,16 +1806,18 @@
         <x:v>Inventoried</x:v>
       </x:c>
       <x:c r="H31" s="4" t="str">
-        <x:v>Not Tested</x:v>
+        <x:v>Tested</x:v>
       </x:c>
       <x:c r="I31" s="4" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="J31" s="4" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K31" s="1" t="str"/>
-      <x:c r="L31" s="25" t="str"/>
+      <x:c r="K31" s="1"/>
+      <x:c r="L31" s="25" t="str">
+        <x:v>Smoke tested in browser on localhost:4173 with no console errors.</x:v>
+      </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="26" t="str">
@@ -1832,16 +1842,18 @@
         <x:v>Inventoried</x:v>
       </x:c>
       <x:c r="H32" s="4" t="str">
-        <x:v>Not Tested</x:v>
+        <x:v>Tested</x:v>
       </x:c>
       <x:c r="I32" s="4" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="J32" s="4" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K32" s="1" t="str"/>
-      <x:c r="L32" s="25" t="str"/>
+      <x:c r="K32" s="1"/>
+      <x:c r="L32" s="25" t="str">
+        <x:v>Smoke tested in browser on localhost:4173 with no console errors.</x:v>
+      </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="26" t="str">
@@ -1874,8 +1886,8 @@
       <x:c r="J33" s="4" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K33" s="1" t="str"/>
-      <x:c r="L33" s="25" t="str"/>
+      <x:c r="K33" s="1"/>
+      <x:c r="L33" s="25"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="26" t="str">
@@ -1908,8 +1920,8 @@
       <x:c r="J34" s="4" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K34" s="1" t="str"/>
-      <x:c r="L34" s="25" t="str"/>
+      <x:c r="K34" s="1"/>
+      <x:c r="L34" s="25"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="26" t="str">
@@ -1942,8 +1954,8 @@
       <x:c r="J35" s="4" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K35" s="1" t="str"/>
-      <x:c r="L35" s="25" t="str"/>
+      <x:c r="K35" s="1"/>
+      <x:c r="L35" s="25"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="26" t="str">
@@ -1976,8 +1988,8 @@
       <x:c r="J36" s="4" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K36" s="1" t="str"/>
-      <x:c r="L36" s="25" t="str"/>
+      <x:c r="K36" s="1"/>
+      <x:c r="L36" s="25"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="26" t="str">
@@ -2010,8 +2022,8 @@
       <x:c r="J37" s="4" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K37" s="1" t="str"/>
-      <x:c r="L37" s="25" t="str"/>
+      <x:c r="K37" s="1"/>
+      <x:c r="L37" s="25"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="26" t="str">
@@ -2044,8 +2056,8 @@
       <x:c r="J38" s="4" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K38" s="1" t="str"/>
-      <x:c r="L38" s="25" t="str"/>
+      <x:c r="K38" s="1"/>
+      <x:c r="L38" s="25"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="26" t="str">
@@ -2078,8 +2090,8 @@
       <x:c r="J39" s="4" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K39" s="1" t="str"/>
-      <x:c r="L39" s="25" t="str"/>
+      <x:c r="K39" s="1"/>
+      <x:c r="L39" s="25"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="26" t="str">
@@ -2112,8 +2124,8 @@
       <x:c r="J40" s="4" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K40" s="1" t="str"/>
-      <x:c r="L40" s="25" t="str"/>
+      <x:c r="K40" s="1"/>
+      <x:c r="L40" s="25"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="26" t="str">
@@ -2146,8 +2158,8 @@
       <x:c r="J41" s="4" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K41" s="1" t="str"/>
-      <x:c r="L41" s="25" t="str"/>
+      <x:c r="K41" s="1"/>
+      <x:c r="L41" s="25"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="26" t="str">
@@ -2180,8 +2192,8 @@
       <x:c r="J42" s="4" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K42" s="1" t="str"/>
-      <x:c r="L42" s="25" t="str"/>
+      <x:c r="K42" s="1"/>
+      <x:c r="L42" s="25"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="26" t="str">
@@ -2214,8 +2226,8 @@
       <x:c r="J43" s="4" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="K43" s="1" t="str"/>
-      <x:c r="L43" s="25" t="str"/>
+      <x:c r="K43" s="1"/>
+      <x:c r="L43" s="25"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="26" t="str">
@@ -2248,8 +2260,8 @@
       <x:c r="J44" s="4" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="K44" s="1" t="str"/>
-      <x:c r="L44" s="25" t="str"/>
+      <x:c r="K44" s="1"/>
+      <x:c r="L44" s="25"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="26" t="str">
@@ -2282,8 +2294,8 @@
       <x:c r="J45" s="4" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="K45" s="1" t="str"/>
-      <x:c r="L45" s="25" t="str"/>
+      <x:c r="K45" s="1"/>
+      <x:c r="L45" s="25"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="26" t="str">
@@ -2316,8 +2328,8 @@
       <x:c r="J46" s="4" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="K46" s="1" t="str"/>
-      <x:c r="L46" s="25" t="str"/>
+      <x:c r="K46" s="1"/>
+      <x:c r="L46" s="25"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="26" t="str">
@@ -2350,8 +2362,8 @@
       <x:c r="J47" s="4" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="K47" s="1" t="str"/>
-      <x:c r="L47" s="25" t="str"/>
+      <x:c r="K47" s="1"/>
+      <x:c r="L47" s="25"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="26" t="str">
@@ -2376,16 +2388,18 @@
         <x:v>Inventoried</x:v>
       </x:c>
       <x:c r="H48" s="4" t="str">
-        <x:v>Not Tested</x:v>
+        <x:v>Tested</x:v>
       </x:c>
       <x:c r="I48" s="4" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="J48" s="4" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="K48" s="1" t="str"/>
-      <x:c r="L48" s="25" t="str"/>
+      <x:c r="K48" s="1"/>
+      <x:c r="L48" s="25" t="str">
+        <x:v>Smoke tested in browser on localhost:4173 with no console errors.</x:v>
+      </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="26" t="str">
@@ -2410,16 +2424,18 @@
         <x:v>Inventoried</x:v>
       </x:c>
       <x:c r="H49" s="4" t="str">
-        <x:v>Not Tested</x:v>
+        <x:v>Tested</x:v>
       </x:c>
       <x:c r="I49" s="4" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="J49" s="4" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="K49" s="1" t="str"/>
-      <x:c r="L49" s="25" t="str"/>
+      <x:c r="K49" s="1"/>
+      <x:c r="L49" s="25" t="str">
+        <x:v>Smoke tested in browser on localhost:4173 with no console errors.</x:v>
+      </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="26" t="str">
@@ -2452,8 +2468,8 @@
       <x:c r="J50" s="4" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="K50" s="1" t="str"/>
-      <x:c r="L50" s="25" t="str"/>
+      <x:c r="K50" s="1"/>
+      <x:c r="L50" s="25"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="26" t="str">
@@ -2478,16 +2494,18 @@
         <x:v>Inventoried</x:v>
       </x:c>
       <x:c r="H51" s="4" t="str">
-        <x:v>Not Tested</x:v>
+        <x:v>Tested</x:v>
       </x:c>
       <x:c r="I51" s="4" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="J51" s="4" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="K51" s="1" t="str"/>
-      <x:c r="L51" s="25" t="str"/>
+      <x:c r="K51" s="1"/>
+      <x:c r="L51" s="25" t="str">
+        <x:v>Smoke tested in browser on localhost:4173 with no console errors.</x:v>
+      </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="26" t="str">
@@ -2520,8 +2538,8 @@
       <x:c r="J52" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K52" s="1" t="str"/>
-      <x:c r="L52" s="25" t="str"/>
+      <x:c r="K52" s="1"/>
+      <x:c r="L52" s="25"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="26" t="str">
@@ -2554,8 +2572,8 @@
       <x:c r="J53" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K53" s="1" t="str"/>
-      <x:c r="L53" s="25" t="str"/>
+      <x:c r="K53" s="1"/>
+      <x:c r="L53" s="25"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="26" t="str">
@@ -2588,8 +2606,8 @@
       <x:c r="J54" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K54" s="1" t="str"/>
-      <x:c r="L54" s="25" t="str"/>
+      <x:c r="K54" s="1"/>
+      <x:c r="L54" s="25"/>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="26" t="str">
@@ -2622,8 +2640,8 @@
       <x:c r="J55" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K55" s="1" t="str"/>
-      <x:c r="L55" s="25" t="str"/>
+      <x:c r="K55" s="1"/>
+      <x:c r="L55" s="25"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="26" t="str">
@@ -2656,8 +2674,8 @@
       <x:c r="J56" s="4" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K56" s="1" t="str"/>
-      <x:c r="L56" s="25" t="str"/>
+      <x:c r="K56" s="1"/>
+      <x:c r="L56" s="25"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="26" t="str">
@@ -2690,8 +2708,8 @@
       <x:c r="J57" s="4" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K57" s="1" t="str"/>
-      <x:c r="L57" s="25" t="str"/>
+      <x:c r="K57" s="1"/>
+      <x:c r="L57" s="25"/>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="26" t="str">
@@ -2724,8 +2742,8 @@
       <x:c r="J58" s="4" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K58" s="1" t="str"/>
-      <x:c r="L58" s="25" t="str"/>
+      <x:c r="K58" s="1"/>
+      <x:c r="L58" s="25"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="26" t="str">
@@ -2758,8 +2776,8 @@
       <x:c r="J59" s="4" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K59" s="1" t="str"/>
-      <x:c r="L59" s="25" t="str"/>
+      <x:c r="K59" s="1"/>
+      <x:c r="L59" s="25"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="26" t="str">
@@ -2792,8 +2810,8 @@
       <x:c r="J60" s="4" t="str">
         <x:v>P1</x:v>
       </x:c>
-      <x:c r="K60" s="1" t="str"/>
-      <x:c r="L60" s="25" t="str"/>
+      <x:c r="K60" s="1"/>
+      <x:c r="L60" s="25"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="26" t="str">
@@ -2826,8 +2844,8 @@
       <x:c r="J61" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K61" s="1" t="str"/>
-      <x:c r="L61" s="25" t="str"/>
+      <x:c r="K61" s="1"/>
+      <x:c r="L61" s="25"/>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="26" t="str">
@@ -2860,8 +2878,8 @@
       <x:c r="J62" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K62" s="1" t="str"/>
-      <x:c r="L62" s="25" t="str"/>
+      <x:c r="K62" s="1"/>
+      <x:c r="L62" s="25"/>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="26" t="str">
@@ -2894,8 +2912,8 @@
       <x:c r="J63" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K63" s="1" t="str"/>
-      <x:c r="L63" s="25" t="str"/>
+      <x:c r="K63" s="1"/>
+      <x:c r="L63" s="25"/>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="26" t="str">
@@ -2928,8 +2946,8 @@
       <x:c r="J64" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K64" s="1" t="str"/>
-      <x:c r="L64" s="25" t="str"/>
+      <x:c r="K64" s="1"/>
+      <x:c r="L64" s="25"/>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="26" t="str">
@@ -2962,8 +2980,8 @@
       <x:c r="J65" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K65" s="1" t="str"/>
-      <x:c r="L65" s="25" t="str"/>
+      <x:c r="K65" s="1"/>
+      <x:c r="L65" s="25"/>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="26" t="str">
@@ -2996,8 +3014,8 @@
       <x:c r="J66" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K66" s="1" t="str"/>
-      <x:c r="L66" s="25" t="str"/>
+      <x:c r="K66" s="1"/>
+      <x:c r="L66" s="25"/>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="26" t="str">
@@ -3030,8 +3048,8 @@
       <x:c r="J67" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K67" s="1" t="str"/>
-      <x:c r="L67" s="25" t="str"/>
+      <x:c r="K67" s="1"/>
+      <x:c r="L67" s="25"/>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="26" t="str">
@@ -3064,8 +3082,8 @@
       <x:c r="J68" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K68" s="1" t="str"/>
-      <x:c r="L68" s="25" t="str"/>
+      <x:c r="K68" s="1"/>
+      <x:c r="L68" s="25"/>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="26" t="str">
@@ -3098,8 +3116,8 @@
       <x:c r="J69" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K69" s="1" t="str"/>
-      <x:c r="L69" s="25" t="str"/>
+      <x:c r="K69" s="1"/>
+      <x:c r="L69" s="25"/>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="26" t="str">
@@ -3132,8 +3150,8 @@
       <x:c r="J70" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K70" s="1" t="str"/>
-      <x:c r="L70" s="25" t="str"/>
+      <x:c r="K70" s="1"/>
+      <x:c r="L70" s="25"/>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="26" t="str">
@@ -3166,8 +3184,8 @@
       <x:c r="J71" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K71" s="1" t="str"/>
-      <x:c r="L71" s="25" t="str"/>
+      <x:c r="K71" s="1"/>
+      <x:c r="L71" s="25"/>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="26" t="str">
@@ -3200,8 +3218,8 @@
       <x:c r="J72" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K72" s="1" t="str"/>
-      <x:c r="L72" s="25" t="str"/>
+      <x:c r="K72" s="1"/>
+      <x:c r="L72" s="25"/>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="26" t="str">
@@ -3234,8 +3252,8 @@
       <x:c r="J73" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K73" s="1" t="str"/>
-      <x:c r="L73" s="25" t="str"/>
+      <x:c r="K73" s="1"/>
+      <x:c r="L73" s="25"/>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="26" t="str">
@@ -3268,8 +3286,8 @@
       <x:c r="J74" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K74" s="1" t="str"/>
-      <x:c r="L74" s="25" t="str"/>
+      <x:c r="K74" s="1"/>
+      <x:c r="L74" s="25"/>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="26" t="str">
@@ -3302,8 +3320,8 @@
       <x:c r="J75" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K75" s="1" t="str"/>
-      <x:c r="L75" s="25" t="str"/>
+      <x:c r="K75" s="1"/>
+      <x:c r="L75" s="25"/>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="26" t="str">
@@ -3336,8 +3354,8 @@
       <x:c r="J76" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K76" s="1" t="str"/>
-      <x:c r="L76" s="25" t="str"/>
+      <x:c r="K76" s="1"/>
+      <x:c r="L76" s="25"/>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="26" t="str">
@@ -3370,8 +3388,8 @@
       <x:c r="J77" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K77" s="1" t="str"/>
-      <x:c r="L77" s="25" t="str"/>
+      <x:c r="K77" s="1"/>
+      <x:c r="L77" s="25"/>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="26" t="str">
@@ -3404,8 +3422,8 @@
       <x:c r="J78" s="4" t="str">
         <x:v>P3</x:v>
       </x:c>
-      <x:c r="K78" s="1" t="str"/>
-      <x:c r="L78" s="25" t="str"/>
+      <x:c r="K78" s="1"/>
+      <x:c r="L78" s="25"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="26" t="str">
@@ -3438,8 +3456,8 @@
       <x:c r="J79" s="4" t="str">
         <x:v>P3</x:v>
       </x:c>
-      <x:c r="K79" s="1" t="str"/>
-      <x:c r="L79" s="25" t="str"/>
+      <x:c r="K79" s="1"/>
+      <x:c r="L79" s="25"/>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="26" t="str">
@@ -3472,8 +3490,8 @@
       <x:c r="J80" s="4" t="str">
         <x:v>P3</x:v>
       </x:c>
-      <x:c r="K80" s="1" t="str"/>
-      <x:c r="L80" s="25" t="str"/>
+      <x:c r="K80" s="1"/>
+      <x:c r="L80" s="25"/>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="26" t="str">
@@ -3506,8 +3524,8 @@
       <x:c r="J81" s="4" t="str">
         <x:v>P3</x:v>
       </x:c>
-      <x:c r="K81" s="1" t="str"/>
-      <x:c r="L81" s="25" t="str"/>
+      <x:c r="K81" s="1"/>
+      <x:c r="L81" s="25"/>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="26" t="str">
@@ -3540,8 +3558,8 @@
       <x:c r="J82" s="4" t="str">
         <x:v>P3</x:v>
       </x:c>
-      <x:c r="K82" s="1" t="str"/>
-      <x:c r="L82" s="25" t="str"/>
+      <x:c r="K82" s="1"/>
+      <x:c r="L82" s="25"/>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="35" t="str">
@@ -3574,8 +3592,8 @@
       <x:c r="J83" s="36" t="str">
         <x:v>P3</x:v>
       </x:c>
-      <x:c r="K83" s="30" t="str"/>
-      <x:c r="L83" s="31" t="str"/>
+      <x:c r="K83" s="30"/>
+      <x:c r="L83" s="31"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="4">
@@ -3594,7 +3612,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R781b93c0ecfa4eba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16ce7ac7ef304d0a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3655,171 +3673,279 @@
       <x:c r="A2" s="26" t="str">
         <x:v>TR-001</x:v>
       </x:c>
-      <x:c r="B2" s="1" t="str"/>
-      <x:c r="C2" s="1" t="str"/>
+      <x:c r="B2" s="1" t="str">
+        <x:v>BF-003</x:v>
+      </x:c>
+      <x:c r="C2" s="1" t="str">
+        <x:v>2026-06-21</x:v>
+      </x:c>
       <x:c r="D2" s="1" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="E2" s="1" t="str"/>
-      <x:c r="F2" s="1" t="str"/>
-      <x:c r="G2" s="1" t="str"/>
+      <x:c r="E2" s="1" t="str">
+        <x:v>Open http://localhost:4173/timer.html.</x:v>
+      </x:c>
+      <x:c r="F2" s="1" t="str">
+        <x:v>BellForge Timer loads with timer workspace, Workouts tab, ready timer, and no console errors.</x:v>
+      </x:c>
+      <x:c r="G2" s="1" t="str">
+        <x:v>Loaded with title BellForge Timer, Workouts active, timer Ready, 13 workout rows, 75 exercise cards, no console errors.</x:v>
+      </x:c>
       <x:c r="H2" s="1" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="I2" s="1" t="str"/>
-      <x:c r="J2" s="1" t="str"/>
+      <x:c r="J2" s="1" t="str">
+        <x:v>Browser smoke test output</x:v>
+      </x:c>
       <x:c r="K2" s="25" t="str"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="26" t="str">
         <x:v>TR-002</x:v>
       </x:c>
-      <x:c r="B3" s="1" t="str"/>
-      <x:c r="C3" s="1" t="str"/>
+      <x:c r="B3" s="1" t="str">
+        <x:v>BF-004</x:v>
+      </x:c>
+      <x:c r="C3" s="1" t="str">
+        <x:v>2026-06-21</x:v>
+      </x:c>
       <x:c r="D3" s="1" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="E3" s="1" t="str"/>
-      <x:c r="F3" s="1" t="str"/>
-      <x:c r="G3" s="1" t="str"/>
+      <x:c r="E3" s="1" t="str">
+        <x:v>Click Workouts, select workout, click Equipment.</x:v>
+      </x:c>
+      <x:c r="F3" s="1" t="str">
+        <x:v>Tabs switch active button and visible panel without losing timer context.</x:v>
+      </x:c>
+      <x:c r="G3" s="1" t="str">
+        <x:v>Visible panel changed from templates to moves to equipment; selected workout/timer context remained.</x:v>
+      </x:c>
       <x:c r="H3" s="1" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="I3" s="1" t="str"/>
-      <x:c r="J3" s="1" t="str"/>
+      <x:c r="J3" s="1" t="str">
+        <x:v>Browser smoke test output</x:v>
+      </x:c>
       <x:c r="K3" s="25" t="str"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="26" t="str">
         <x:v>TR-003</x:v>
       </x:c>
-      <x:c r="B4" s="1" t="str"/>
-      <x:c r="C4" s="1" t="str"/>
+      <x:c r="B4" s="1" t="str">
+        <x:v>BF-020</x:v>
+      </x:c>
+      <x:c r="C4" s="1" t="str">
+        <x:v>2026-06-21</x:v>
+      </x:c>
       <x:c r="D4" s="1" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="E4" s="1" t="str"/>
-      <x:c r="F4" s="1" t="str"/>
-      <x:c r="G4" s="1" t="str"/>
+      <x:c r="E4" s="1" t="str">
+        <x:v>Open Workouts tab.</x:v>
+      </x:c>
+      <x:c r="F4" s="1" t="str">
+        <x:v>Predefined and custom workouts render in list.</x:v>
+      </x:c>
+      <x:c r="G4" s="1" t="str">
+        <x:v>Workouts panel showed 13 template rows.</x:v>
+      </x:c>
       <x:c r="H4" s="1" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="I4" s="1" t="str"/>
-      <x:c r="J4" s="1" t="str"/>
+      <x:c r="J4" s="1" t="str">
+        <x:v>Browser smoke test output</x:v>
+      </x:c>
       <x:c r="K4" s="25" t="str"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="26" t="str">
         <x:v>TR-004</x:v>
       </x:c>
-      <x:c r="B5" s="1" t="str"/>
-      <x:c r="C5" s="1" t="str"/>
+      <x:c r="B5" s="1" t="str">
+        <x:v>BF-022</x:v>
+      </x:c>
+      <x:c r="C5" s="1" t="str">
+        <x:v>2026-06-21</x:v>
+      </x:c>
       <x:c r="D5" s="1" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="E5" s="1" t="str"/>
-      <x:c r="F5" s="1" t="str"/>
-      <x:c r="G5" s="1" t="str"/>
+      <x:c r="E5" s="1" t="str">
+        <x:v>Select Muscle Gain: Full Body workout.</x:v>
+      </x:c>
+      <x:c r="F5" s="1" t="str">
+        <x:v>Timer config updates to selected workout and switches to Exercises.</x:v>
+      </x:c>
+      <x:c r="G5" s="1" t="str">
+        <x:v>Active tab became Exercises; selected workout Muscle Gain: Full Body; round label Round 1 of 32; movement Goblet Squat.</x:v>
+      </x:c>
       <x:c r="H5" s="1" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="I5" s="1" t="str"/>
-      <x:c r="J5" s="1" t="str"/>
+      <x:c r="J5" s="1" t="str">
+        <x:v>Browser smoke test output</x:v>
+      </x:c>
       <x:c r="K5" s="25" t="str"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="26" t="str">
         <x:v>TR-005</x:v>
       </x:c>
-      <x:c r="B6" s="1" t="str"/>
-      <x:c r="C6" s="1" t="str"/>
+      <x:c r="B6" s="1" t="str">
+        <x:v>BF-050</x:v>
+      </x:c>
+      <x:c r="C6" s="1" t="str">
+        <x:v>2026-06-21</x:v>
+      </x:c>
       <x:c r="D6" s="1" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="E6" s="1" t="str"/>
-      <x:c r="F6" s="1" t="str"/>
-      <x:c r="G6" s="1" t="str"/>
+      <x:c r="E6" s="1" t="str">
+        <x:v>After selecting Muscle Gain: Full Body, inspect selected workout schedule state.</x:v>
+      </x:c>
+      <x:c r="F6" s="1" t="str">
+        <x:v>Selected workout schedule reflects chosen workout and active movement.</x:v>
+      </x:c>
+      <x:c r="G6" s="1" t="str">
+        <x:v>Selected workout title Muscle Gain: Full Body and current movement Goblet Squat were visible.</x:v>
+      </x:c>
       <x:c r="H6" s="1" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="I6" s="1" t="str"/>
-      <x:c r="J6" s="1" t="str"/>
+      <x:c r="J6" s="1" t="str">
+        <x:v>Browser smoke test output</x:v>
+      </x:c>
       <x:c r="K6" s="25" t="str"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="26" t="str">
         <x:v>TR-006</x:v>
       </x:c>
-      <x:c r="B7" s="1" t="str"/>
-      <x:c r="C7" s="1" t="str"/>
+      <x:c r="B7" s="1" t="str">
+        <x:v>BF-047</x:v>
+      </x:c>
+      <x:c r="C7" s="1" t="str">
+        <x:v>2026-06-21</x:v>
+      </x:c>
       <x:c r="D7" s="1" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="E7" s="1" t="str"/>
-      <x:c r="F7" s="1" t="str"/>
-      <x:c r="G7" s="1" t="str"/>
+      <x:c r="E7" s="1" t="str">
+        <x:v>Load app and inspect Exercises data.</x:v>
+      </x:c>
+      <x:c r="F7" s="1" t="str">
+        <x:v>Exercise library renders deduped exercise cards.</x:v>
+      </x:c>
+      <x:c r="G7" s="1" t="str">
+        <x:v>Exercise library showed 75 result cards on load.</x:v>
+      </x:c>
       <x:c r="H7" s="1" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="I7" s="1" t="str"/>
-      <x:c r="J7" s="1" t="str"/>
+      <x:c r="J7" s="1" t="str">
+        <x:v>Browser smoke test output</x:v>
+      </x:c>
       <x:c r="K7" s="25" t="str"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="26" t="str">
         <x:v>TR-007</x:v>
       </x:c>
-      <x:c r="B8" s="1" t="str"/>
-      <x:c r="C8" s="1" t="str"/>
+      <x:c r="B8" s="1" t="str">
+        <x:v>BF-048</x:v>
+      </x:c>
+      <x:c r="C8" s="1" t="str">
+        <x:v>2026-06-21</x:v>
+      </x:c>
       <x:c r="D8" s="1" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="E8" s="1" t="str"/>
-      <x:c r="F8" s="1" t="str"/>
-      <x:c r="G8" s="1" t="str"/>
+      <x:c r="E8" s="1" t="str">
+        <x:v>Type squat in exercise search.</x:v>
+      </x:c>
+      <x:c r="F8" s="1" t="str">
+        <x:v>Exercise cards filter by search term.</x:v>
+      </x:c>
+      <x:c r="G8" s="1" t="str">
+        <x:v>Exercise results changed from 75 to 6 results for squat.</x:v>
+      </x:c>
       <x:c r="H8" s="1" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="I8" s="1" t="str"/>
-      <x:c r="J8" s="1" t="str"/>
+      <x:c r="J8" s="1" t="str">
+        <x:v>Browser smoke test output</x:v>
+      </x:c>
       <x:c r="K8" s="25" t="str"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="26" t="str">
         <x:v>TR-008</x:v>
       </x:c>
-      <x:c r="B9" s="1" t="str"/>
-      <x:c r="C9" s="1" t="str"/>
+      <x:c r="B9" s="1" t="str">
+        <x:v>BF-030</x:v>
+      </x:c>
+      <x:c r="C9" s="1" t="str">
+        <x:v>2026-06-21</x:v>
+      </x:c>
       <x:c r="D9" s="1" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="E9" s="1" t="str"/>
-      <x:c r="F9" s="1" t="str"/>
-      <x:c r="G9" s="1" t="str"/>
+      <x:c r="E9" s="1" t="str">
+        <x:v>Open Equipment tab.</x:v>
+      </x:c>
+      <x:c r="F9" s="1" t="str">
+        <x:v>Equipment list and selected count render.</x:v>
+      </x:c>
+      <x:c r="G9" s="1" t="str">
+        <x:v>Equipment tab showed 4 selected before interaction.</x:v>
+      </x:c>
       <x:c r="H9" s="1" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="I9" s="1" t="str"/>
-      <x:c r="J9" s="1" t="str"/>
+      <x:c r="J9" s="1" t="str">
+        <x:v>Browser smoke test output</x:v>
+      </x:c>
       <x:c r="K9" s="25" t="str"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="26" t="str">
         <x:v>TR-009</x:v>
       </x:c>
-      <x:c r="B10" s="1" t="str"/>
-      <x:c r="C10" s="1" t="str"/>
+      <x:c r="B10" s="1" t="str">
+        <x:v>BF-031</x:v>
+      </x:c>
+      <x:c r="C10" s="1" t="str">
+        <x:v>2026-06-21</x:v>
+      </x:c>
       <x:c r="D10" s="1" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="E10" s="1" t="str"/>
-      <x:c r="F10" s="1" t="str"/>
-      <x:c r="G10" s="1" t="str"/>
+      <x:c r="E10" s="1" t="str">
+        <x:v>Toggle Bodyweight equipment off and back on.</x:v>
+      </x:c>
+      <x:c r="F10" s="1" t="str">
+        <x:v>Selected count changes and can be restored.</x:v>
+      </x:c>
+      <x:c r="G10" s="1" t="str">
+        <x:v>Selected count changed 4 -&gt; 3 -&gt; 4.</x:v>
+      </x:c>
       <x:c r="H10" s="1" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="I10" s="1" t="str"/>
-      <x:c r="J10" s="1" t="str"/>
+      <x:c r="J10" s="1" t="str">
+        <x:v>Browser smoke test output</x:v>
+      </x:c>
       <x:c r="K10" s="25" t="str"/>
     </x:row>
     <x:row r="11">
@@ -5559,7 +5685,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad1d4fad64554935"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Radc15d85ce4f41d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7431,7 +7557,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8768b6fb8c6a4201"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb445877edb448e1"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Restore manual timer setup
</commit_message>
<xml_diff>
--- a/docs/qa/bellforge-feature-tracker.xlsx
+++ b/docs/qa/bellforge-feature-tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rde54910d3a1f4e51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Stories" sheetId="2" r:id="Re1002ef8d6f34d04"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Runs" sheetId="3" r:id="R620b7ece0c594eaf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defects" sheetId="4" r:id="R22c105b773cd4e5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="5" r:id="Re8e4d6e118b847d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R6dd674ecadd74220"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Stories" sheetId="2" r:id="Ra5668fd6517e4948"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Runs" sheetId="3" r:id="R7ced599b78b8493a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defects" sheetId="4" r:id="Rfda6aec658b94f29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="5" r:id="R03c9c2057f8d4095"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -559,7 +559,7 @@
       </x:c>
       <x:c r="B6" s="4" t="n">
         <x:f>COUNTIF('Feature Stories'!H2:H83,"Not Tested")</x:f>
-        <x:v>73</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="C6" s="1"/>
       <x:c r="D6" s="1"/>
@@ -952,16 +952,20 @@
         <x:v>Inventoried</x:v>
       </x:c>
       <x:c r="H6" s="4" t="str">
-        <x:v>Not Tested</x:v>
+        <x:v>Retested</x:v>
       </x:c>
       <x:c r="I6" s="4" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="J6" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K6" s="1"/>
-      <x:c r="L6" s="25"/>
+      <x:c r="K6" s="1" t="str">
+        <x:v>BUG-001</x:v>
+      </x:c>
+      <x:c r="L6" s="25" t="str">
+        <x:v>Retested after compact Manual setup drawer fix; fields are visible/reachable and validation works.</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="26" t="str">
@@ -977,7 +981,7 @@
         <x:v>As a user, I want to set workout rounds so the timer duration matches the planned EMOM.</x:v>
       </x:c>
       <x:c r="E7" s="1" t="str">
-        <x:v>Rounds are normalized to at least 1; total duration is rounds * 60 seconds.</x:v>
+        <x:v>Rounds are normalized to at least 1; total duration is rounds * 60 minus the final rest interval.</x:v>
       </x:c>
       <x:c r="F7" s="1" t="str">
         <x:v>timer.html; timer.js normalizeRounds; timer.js getPlannedDurationSeconds</x:v>
@@ -986,16 +990,20 @@
         <x:v>Inventoried</x:v>
       </x:c>
       <x:c r="H7" s="4" t="str">
-        <x:v>Not Tested</x:v>
+        <x:v>Retested</x:v>
       </x:c>
       <x:c r="I7" s="4" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="J7" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K7" s="1"/>
-      <x:c r="L7" s="25"/>
+      <x:c r="K7" s="1" t="str">
+        <x:v>BUG-001</x:v>
+      </x:c>
+      <x:c r="L7" s="25" t="str">
+        <x:v>Retested after compact Manual setup drawer fix; fields are visible/reachable and validation works.</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="26" t="str">
@@ -1020,16 +1028,20 @@
         <x:v>Inventoried</x:v>
       </x:c>
       <x:c r="H8" s="4" t="str">
-        <x:v>Not Tested</x:v>
+        <x:v>Retested</x:v>
       </x:c>
       <x:c r="I8" s="4" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="J8" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K8" s="1"/>
-      <x:c r="L8" s="25"/>
+      <x:c r="K8" s="1" t="str">
+        <x:v>BUG-001</x:v>
+      </x:c>
+      <x:c r="L8" s="25" t="str">
+        <x:v>Retested after compact Manual setup drawer fix; fields are visible/reachable and validation works.</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="26" t="str">
@@ -1088,16 +1100,18 @@
         <x:v>Inventoried</x:v>
       </x:c>
       <x:c r="H10" s="4" t="str">
-        <x:v>Not Tested</x:v>
+        <x:v>Tested</x:v>
       </x:c>
       <x:c r="I10" s="4" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="J10" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="K10" s="1"/>
-      <x:c r="L10" s="25"/>
+      <x:c r="L10" s="25" t="str">
+        <x:v>Visible control smoke tested in browser on localhost:4173.</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="26" t="str">
@@ -1122,16 +1136,18 @@
         <x:v>Inventoried</x:v>
       </x:c>
       <x:c r="H11" s="4" t="str">
-        <x:v>Not Tested</x:v>
+        <x:v>Tested</x:v>
       </x:c>
       <x:c r="I11" s="4" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="J11" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="K11" s="1"/>
-      <x:c r="L11" s="25"/>
+      <x:c r="L11" s="25" t="str">
+        <x:v>Visible control smoke tested in browser on localhost:4173.</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="26" t="str">
@@ -1156,16 +1172,18 @@
         <x:v>Inventoried</x:v>
       </x:c>
       <x:c r="H12" s="4" t="str">
-        <x:v>Not Tested</x:v>
+        <x:v>Tested</x:v>
       </x:c>
       <x:c r="I12" s="4" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="J12" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="K12" s="1"/>
-      <x:c r="L12" s="25"/>
+      <x:c r="L12" s="25" t="str">
+        <x:v>Visible control smoke tested in browser on localhost:4173.</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="26" t="str">
@@ -1215,7 +1233,7 @@
         <x:v>As a trainee, I want the workout to end when all active work is done so I do not sit through an unnecessary final rest.</x:v>
       </x:c>
       <x:c r="E14" s="1" t="str">
-        <x:v>Timer snapshot reaches total duration and running status calls completeWorkout; total duration is rounds * 60 with work/rest inside each round.</x:v>
+        <x:v>Timer completes when final active work interval ends, so the last rest interval is skipped.</x:v>
       </x:c>
       <x:c r="F14" s="1" t="str">
         <x:v>app.js updateDisplay; timer.js getTimerSnapshot</x:v>
@@ -1258,16 +1276,18 @@
         <x:v>Inventoried</x:v>
       </x:c>
       <x:c r="H15" s="4" t="str">
-        <x:v>Not Tested</x:v>
+        <x:v>Tested</x:v>
       </x:c>
       <x:c r="I15" s="4" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="J15" s="4" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="K15" s="1"/>
-      <x:c r="L15" s="25"/>
+      <x:c r="K15" s="1" t="str"/>
+      <x:c r="L15" s="25" t="str">
+        <x:v>Retested with 2 rounds, 1s work / 59s rest; rest-mode activated between active rounds.</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="26" t="str">
@@ -1326,16 +1346,18 @@
         <x:v>Inventoried</x:v>
       </x:c>
       <x:c r="H17" s="4" t="str">
-        <x:v>Not Tested</x:v>
+        <x:v>Tested</x:v>
       </x:c>
       <x:c r="I17" s="4" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="J17" s="4" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="K17" s="1"/>
-      <x:c r="L17" s="25"/>
+      <x:c r="L17" s="25" t="str">
+        <x:v>Visible control smoke tested in browser on localhost:4173.</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="26" t="str">
@@ -3612,7 +3634,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16ce7ac7ef304d0a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8362857c808648aa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3952,209 +3974,353 @@
       <x:c r="A11" s="26" t="str">
         <x:v>TR-010</x:v>
       </x:c>
-      <x:c r="B11" s="1" t="str"/>
-      <x:c r="C11" s="1" t="str"/>
+      <x:c r="B11" s="1" t="str">
+        <x:v>BF-016</x:v>
+      </x:c>
+      <x:c r="C11" s="1" t="str">
+        <x:v>2026-06-21</x:v>
+      </x:c>
       <x:c r="D11" s="1" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="E11" s="1" t="str"/>
-      <x:c r="F11" s="1" t="str"/>
-      <x:c r="G11" s="1" t="str"/>
+      <x:c r="E11" s="1" t="str">
+        <x:v>Click Sound On, then click Sound Off to restore.</x:v>
+      </x:c>
+      <x:c r="F11" s="1" t="str">
+        <x:v>Button toggles text and aria-pressed without console errors.</x:v>
+      </x:c>
+      <x:c r="G11" s="1" t="str">
+        <x:v>Sound On -&gt; Sound Off -&gt; Sound On; aria-pressed false after disabling.</x:v>
+      </x:c>
       <x:c r="H11" s="1" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="I11" s="1" t="str"/>
-      <x:c r="J11" s="1" t="str"/>
+      <x:c r="J11" s="1" t="str">
+        <x:v>Browser timer-control output</x:v>
+      </x:c>
       <x:c r="K11" s="25" t="str"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="26" t="str">
         <x:v>TR-011</x:v>
       </x:c>
-      <x:c r="B12" s="1" t="str"/>
-      <x:c r="C12" s="1" t="str"/>
+      <x:c r="B12" s="1" t="str">
+        <x:v>BF-009</x:v>
+      </x:c>
+      <x:c r="C12" s="1" t="str">
+        <x:v>2026-06-21</x:v>
+      </x:c>
       <x:c r="D12" s="1" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="E12" s="1" t="str"/>
-      <x:c r="F12" s="1" t="str"/>
-      <x:c r="G12" s="1" t="str"/>
+      <x:c r="E12" s="1" t="str">
+        <x:v>Click Start on default timer.</x:v>
+      </x:c>
+      <x:c r="F12" s="1" t="str">
+        <x:v>Timer enters Running; Start disables; Pause and Complete enable; elapsed/time left update.</x:v>
+      </x:c>
+      <x:c r="G12" s="1" t="str">
+        <x:v>Running after 1.2s; Start disabled, Pause enabled, Complete enabled, elapsed 00:01, time left 00:29.</x:v>
+      </x:c>
       <x:c r="H12" s="1" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="I12" s="1" t="str"/>
-      <x:c r="J12" s="1" t="str"/>
+      <x:c r="J12" s="1" t="str">
+        <x:v>Browser timer-control output</x:v>
+      </x:c>
       <x:c r="K12" s="25" t="str"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="26" t="str">
         <x:v>TR-012</x:v>
       </x:c>
-      <x:c r="B13" s="1" t="str"/>
-      <x:c r="C13" s="1" t="str"/>
+      <x:c r="B13" s="1" t="str">
+        <x:v>BF-010</x:v>
+      </x:c>
+      <x:c r="C13" s="1" t="str">
+        <x:v>2026-06-21</x:v>
+      </x:c>
       <x:c r="D13" s="1" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="E13" s="1" t="str"/>
-      <x:c r="F13" s="1" t="str"/>
-      <x:c r="G13" s="1" t="str"/>
+      <x:c r="E13" s="1" t="str">
+        <x:v>Click Pause after timer is running.</x:v>
+      </x:c>
+      <x:c r="F13" s="1" t="str">
+        <x:v>Timer enters Paused; Start becomes available; Pause disables.</x:v>
+      </x:c>
+      <x:c r="G13" s="1" t="str">
+        <x:v>Paused with Start enabled and Pause disabled.</x:v>
+      </x:c>
       <x:c r="H13" s="1" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="I13" s="1" t="str"/>
-      <x:c r="J13" s="1" t="str"/>
+      <x:c r="J13" s="1" t="str">
+        <x:v>Browser timer-control output</x:v>
+      </x:c>
       <x:c r="K13" s="25" t="str"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="26" t="str">
         <x:v>TR-013</x:v>
       </x:c>
-      <x:c r="B14" s="1" t="str"/>
-      <x:c r="C14" s="1" t="str"/>
+      <x:c r="B14" s="1" t="str">
+        <x:v>BF-011</x:v>
+      </x:c>
+      <x:c r="C14" s="1" t="str">
+        <x:v>2026-06-21</x:v>
+      </x:c>
       <x:c r="D14" s="1" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="E14" s="1" t="str"/>
-      <x:c r="F14" s="1" t="str"/>
-      <x:c r="G14" s="1" t="str"/>
+      <x:c r="E14" s="1" t="str">
+        <x:v>Click Reset after pausing.</x:v>
+      </x:c>
+      <x:c r="F14" s="1" t="str">
+        <x:v>Timer returns to Ready with elapsed 00:00 and time left 00:30.</x:v>
+      </x:c>
+      <x:c r="G14" s="1" t="str">
+        <x:v>Ready, elapsed 00:00, time left 00:30, Complete disabled.</x:v>
+      </x:c>
       <x:c r="H14" s="1" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="I14" s="1" t="str"/>
-      <x:c r="J14" s="1" t="str"/>
+      <x:c r="J14" s="1" t="str">
+        <x:v>Browser timer-control output</x:v>
+      </x:c>
       <x:c r="K14" s="25" t="str"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="26" t="str">
         <x:v>TR-014</x:v>
       </x:c>
-      <x:c r="B15" s="1" t="str"/>
-      <x:c r="C15" s="1" t="str"/>
+      <x:c r="B15" s="1" t="str">
+        <x:v>BF-005</x:v>
+      </x:c>
+      <x:c r="C15" s="1" t="str">
+        <x:v>2026-06-21</x:v>
+      </x:c>
       <x:c r="D15" s="1" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="E15" s="1" t="str"/>
-      <x:c r="F15" s="1" t="str"/>
-      <x:c r="G15" s="1" t="str"/>
+      <x:c r="E15" s="1" t="str">
+        <x:v>Attempt to fill workout-name as a user-visible control.</x:v>
+      </x:c>
+      <x:c r="F15" s="1" t="str">
+        <x:v>Workout name input should be visible or reachable before starting a manual workout.</x:v>
+      </x:c>
+      <x:c r="G15" s="1" t="str">
+        <x:v>Input exists but computed display is none, width/height are 0, and no setup toggle exists.</x:v>
+      </x:c>
       <x:c r="H15" s="1" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="I15" s="1" t="str"/>
-      <x:c r="J15" s="1" t="str"/>
+        <x:v>Needs UX Fix</x:v>
+      </x:c>
+      <x:c r="I15" s="1" t="str">
+        <x:v>BUG-001</x:v>
+      </x:c>
+      <x:c r="J15" s="1" t="str">
+        <x:v>Browser timer-control output</x:v>
+      </x:c>
       <x:c r="K15" s="25" t="str"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="26" t="str">
         <x:v>TR-015</x:v>
       </x:c>
-      <x:c r="B16" s="1" t="str"/>
-      <x:c r="C16" s="1" t="str"/>
+      <x:c r="B16" s="1" t="str">
+        <x:v>BF-006</x:v>
+      </x:c>
+      <x:c r="C16" s="1" t="str">
+        <x:v>2026-06-21</x:v>
+      </x:c>
       <x:c r="D16" s="1" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="E16" s="1" t="str"/>
-      <x:c r="F16" s="1" t="str"/>
-      <x:c r="G16" s="1" t="str"/>
+      <x:c r="E16" s="1" t="str">
+        <x:v>Attempt to fill rounds as a user-visible control.</x:v>
+      </x:c>
+      <x:c r="F16" s="1" t="str">
+        <x:v>Rounds input should be visible or reachable before starting a manual workout.</x:v>
+      </x:c>
+      <x:c r="G16" s="1" t="str">
+        <x:v>Input exists but computed display is none, width/height are 0, and no setup toggle exists.</x:v>
+      </x:c>
       <x:c r="H16" s="1" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="I16" s="1" t="str"/>
-      <x:c r="J16" s="1" t="str"/>
+        <x:v>Needs UX Fix</x:v>
+      </x:c>
+      <x:c r="I16" s="1" t="str">
+        <x:v>BUG-001</x:v>
+      </x:c>
+      <x:c r="J16" s="1" t="str">
+        <x:v>Browser timer-control output</x:v>
+      </x:c>
       <x:c r="K16" s="25" t="str"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="26" t="str">
         <x:v>TR-016</x:v>
       </x:c>
-      <x:c r="B17" s="1" t="str"/>
-      <x:c r="C17" s="1" t="str"/>
+      <x:c r="B17" s="1" t="str">
+        <x:v>BF-007</x:v>
+      </x:c>
+      <x:c r="C17" s="1" t="str">
+        <x:v>2026-06-21</x:v>
+      </x:c>
       <x:c r="D17" s="1" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="E17" s="1" t="str"/>
-      <x:c r="F17" s="1" t="str"/>
-      <x:c r="G17" s="1" t="str"/>
+      <x:c r="E17" s="1" t="str">
+        <x:v>Attempt to fill work/rest seconds as user-visible controls.</x:v>
+      </x:c>
+      <x:c r="F17" s="1" t="str">
+        <x:v>Work/rest inputs should be visible or reachable and validate work + rest = 60.</x:v>
+      </x:c>
+      <x:c r="G17" s="1" t="str">
+        <x:v>Inputs exist but computed display is none, width/height are 0, and no setup toggle exists.</x:v>
+      </x:c>
       <x:c r="H17" s="1" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="I17" s="1" t="str"/>
-      <x:c r="J17" s="1" t="str"/>
+        <x:v>Needs UX Fix</x:v>
+      </x:c>
+      <x:c r="I17" s="1" t="str">
+        <x:v>BUG-001</x:v>
+      </x:c>
+      <x:c r="J17" s="1" t="str">
+        <x:v>Browser timer-control output</x:v>
+      </x:c>
       <x:c r="K17" s="25" t="str"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="26" t="str">
         <x:v>TR-017</x:v>
       </x:c>
-      <x:c r="B18" s="1" t="str"/>
-      <x:c r="C18" s="1" t="str"/>
+      <x:c r="B18" s="1" t="str">
+        <x:v>BF-005</x:v>
+      </x:c>
+      <x:c r="C18" s="1" t="str">
+        <x:v>2026-06-21</x:v>
+      </x:c>
       <x:c r="D18" s="1" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="E18" s="1" t="str"/>
-      <x:c r="F18" s="1" t="str"/>
-      <x:c r="G18" s="1" t="str"/>
+      <x:c r="E18" s="1" t="str">
+        <x:v>Open Manual setup drawer and fill workout name.</x:v>
+      </x:c>
+      <x:c r="F18" s="1" t="str">
+        <x:v>Workout name is visible/reachable and updates timer title/context.</x:v>
+      </x:c>
+      <x:c r="G18" s="1" t="str">
+        <x:v>Drawer opened; name input was visible 548x48; filling QA Retest Manual updated app title.</x:v>
+      </x:c>
       <x:c r="H18" s="1" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="I18" s="1" t="str"/>
-      <x:c r="J18" s="1" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="I18" s="1" t="str">
+        <x:v>BUG-001</x:v>
+      </x:c>
+      <x:c r="J18" s="1" t="str">
+        <x:v>Browser retest output</x:v>
+      </x:c>
       <x:c r="K18" s="25" t="str"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="26" t="str">
         <x:v>TR-018</x:v>
       </x:c>
-      <x:c r="B19" s="1" t="str"/>
-      <x:c r="C19" s="1" t="str"/>
+      <x:c r="B19" s="1" t="str">
+        <x:v>BF-006</x:v>
+      </x:c>
+      <x:c r="C19" s="1" t="str">
+        <x:v>2026-06-21</x:v>
+      </x:c>
       <x:c r="D19" s="1" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="E19" s="1" t="str"/>
-      <x:c r="F19" s="1" t="str"/>
-      <x:c r="G19" s="1" t="str"/>
+      <x:c r="E19" s="1" t="str">
+        <x:v>Open Manual setup drawer and fill rounds.</x:v>
+      </x:c>
+      <x:c r="F19" s="1" t="str">
+        <x:v>Rounds input is visible/reachable and updates round label/duration.</x:v>
+      </x:c>
+      <x:c r="G19" s="1" t="str">
+        <x:v>Rounds input was visible 176x48; filling 3 updated Round 1 of 3 and context.</x:v>
+      </x:c>
       <x:c r="H19" s="1" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="I19" s="1" t="str"/>
-      <x:c r="J19" s="1" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="I19" s="1" t="str">
+        <x:v>BUG-001</x:v>
+      </x:c>
+      <x:c r="J19" s="1" t="str">
+        <x:v>Browser retest output</x:v>
+      </x:c>
       <x:c r="K19" s="25" t="str"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="26" t="str">
         <x:v>TR-019</x:v>
       </x:c>
-      <x:c r="B20" s="1" t="str"/>
-      <x:c r="C20" s="1" t="str"/>
+      <x:c r="B20" s="1" t="str">
+        <x:v>BF-007</x:v>
+      </x:c>
+      <x:c r="C20" s="1" t="str">
+        <x:v>2026-06-21</x:v>
+      </x:c>
       <x:c r="D20" s="1" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="E20" s="1" t="str"/>
-      <x:c r="F20" s="1" t="str"/>
-      <x:c r="G20" s="1" t="str"/>
+      <x:c r="E20" s="1" t="str">
+        <x:v>Open Manual setup drawer, fill work/rest, then set invalid total.</x:v>
+      </x:c>
+      <x:c r="F20" s="1" t="str">
+        <x:v>Work/rest inputs are visible/reachable; invalid total surfaces validation message.</x:v>
+      </x:c>
+      <x:c r="G20" s="1" t="str">
+        <x:v>40/20 updated context to 40s work / 20s rest; 40/30 produced validation message: Work seconds plus rest seconds must equal 60.</x:v>
+      </x:c>
       <x:c r="H20" s="1" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="I20" s="1" t="str"/>
-      <x:c r="J20" s="1" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="I20" s="1" t="str">
+        <x:v>BUG-001</x:v>
+      </x:c>
+      <x:c r="J20" s="1" t="str">
+        <x:v>Browser retest output</x:v>
+      </x:c>
       <x:c r="K20" s="25" t="str"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="26" t="str">
         <x:v>TR-020</x:v>
       </x:c>
-      <x:c r="B21" s="1" t="str"/>
-      <x:c r="C21" s="1" t="str"/>
+      <x:c r="B21" s="1" t="str">
+        <x:v>BF-014</x:v>
+      </x:c>
+      <x:c r="C21" s="1" t="str">
+        <x:v>2026-06-21</x:v>
+      </x:c>
       <x:c r="D21" s="1" t="str">
         <x:v>Codex</x:v>
       </x:c>
-      <x:c r="E21" s="1" t="str"/>
-      <x:c r="F21" s="1" t="str"/>
-      <x:c r="G21" s="1" t="str"/>
+      <x:c r="E21" s="1" t="str">
+        <x:v>Set 2 rounds, 1s work / 59s rest, start timer and wait 1.5s.</x:v>
+      </x:c>
+      <x:c r="F21" s="1" t="str">
+        <x:v>Rest phase should visually activate between active rounds.</x:v>
+      </x:c>
+      <x:c r="G21" s="1" t="str">
+        <x:v>Timer entered Running Rest phase, body restMode true, Round 1 of 2, 00:59 left.</x:v>
+      </x:c>
       <x:c r="H21" s="1" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="I21" s="1" t="str"/>
-      <x:c r="J21" s="1" t="str"/>
+      <x:c r="J21" s="1" t="str">
+        <x:v>Browser retest output</x:v>
+      </x:c>
       <x:c r="K21" s="25" t="str"/>
     </x:row>
     <x:row r="22">
@@ -5685,7 +5851,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Radc15d85ce4f41d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R106467b7acd74fd4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5750,16 +5916,36 @@
       <x:c r="A2" s="26" t="str">
         <x:v>BUG-001</x:v>
       </x:c>
-      <x:c r="B2" s="1" t="str"/>
-      <x:c r="C2" s="1" t="str"/>
-      <x:c r="D2" s="1" t="str"/>
-      <x:c r="E2" s="1" t="str"/>
-      <x:c r="F2" s="1" t="str"/>
-      <x:c r="G2" s="1" t="str"/>
-      <x:c r="H2" s="1" t="str"/>
-      <x:c r="I2" s="1" t="str"/>
-      <x:c r="J2" s="1" t="str"/>
-      <x:c r="K2" s="1" t="str"/>
+      <x:c r="B2" s="1" t="str">
+        <x:v>BF-005/BF-006/BF-007</x:v>
+      </x:c>
+      <x:c r="C2" s="1" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="D2" s="1" t="str">
+        <x:v>UX</x:v>
+      </x:c>
+      <x:c r="E2" s="1" t="str">
+        <x:v>Manual workout setup fields are hidden and unreachable.</x:v>
+      </x:c>
+      <x:c r="F2" s="1" t="str">
+        <x:v>Browser test found #workout-name, #rounds, #work-seconds, and #rest-seconds exist but all have display:none, width 0, height 0; no setup toggle/button is visible.</x:v>
+      </x:c>
+      <x:c r="G2" s="1" t="str">
+        <x:v>A user should be able to enter or reveal workout name, rounds, work seconds, and rest seconds before starting a manual workout.</x:v>
+      </x:c>
+      <x:c r="H2" s="1" t="str">
+        <x:v>The visible timer panel only exposes Start/Pause/Reset/Sound/Complete, leaving manual setup inaccessible.</x:v>
+      </x:c>
+      <x:c r="I2" s="1" t="str">
+        <x:v>Fixed</x:v>
+      </x:c>
+      <x:c r="J2" s="1" t="str">
+        <x:v>Added compact Manual setup drawer and bumped timer CSS cache key. Pending commit.</x:v>
+      </x:c>
+      <x:c r="K2" s="1" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
       <x:c r="L2" s="25" t="str">
         <x:v>Codex</x:v>
       </x:c>
@@ -7557,7 +7743,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb445877edb448e1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3177dad465b4eae"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>